<commit_message>
Add more checkpoint evaluation Excel results 2
</commit_message>
<xml_diff>
--- a/RL/test_results/eval_dnn_scaled_model_18848453_nato_sc_film_a_gnn_rl_model_3200000_steps.xlsx
+++ b/RL/test_results/eval_dnn_scaled_model_18848453_nato_sc_film_a_gnn_rl_model_3200000_steps.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AV5"/>
+  <dimension ref="A1:AV11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1291,6 +1291,942 @@
         <v>35.32</v>
       </c>
       <c r="AV5" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>1500</v>
+      </c>
+      <c r="B6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>fc_plus_act_8</t>
+        </is>
+      </c>
+      <c r="D6" t="b">
+        <v>1</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1095020</v>
+      </c>
+      <c r="F6" t="n">
+        <v>44.38</v>
+      </c>
+      <c r="G6" t="n">
+        <v>40213</v>
+      </c>
+      <c r="H6" t="n">
+        <v>211.86</v>
+      </c>
+      <c r="I6" t="n">
+        <v>96.33</v>
+      </c>
+      <c r="J6" t="b">
+        <v>0</v>
+      </c>
+      <c r="K6" t="n">
+        <v>40213</v>
+      </c>
+      <c r="L6" t="n">
+        <v>211.86</v>
+      </c>
+      <c r="M6" t="n">
+        <v>96.33</v>
+      </c>
+      <c r="N6" t="b">
+        <v>0</v>
+      </c>
+      <c r="O6" t="b">
+        <v>0</v>
+      </c>
+      <c r="P6" t="n">
+        <v>75</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>75</v>
+      </c>
+      <c r="R6" t="n">
+        <v>20710786.2</v>
+      </c>
+      <c r="S6" t="n">
+        <v>1288.14</v>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>1095020.0|1094175.0|1092243.0|1088359.0|1080459.0|1072559.0|1056561.0|1040563.0|1024763.0|1008963.0|993163.0|977363.0|961365.0|945367.0|929567.0|913767.0|897769.0|881969.0|866169.0|858170.0|850270.0|842370.0|834470.0|826570.0|810572.0|794574.0|778774.0|762974.0|746976.0|731176.0|715376.0|699378.0|683380.0|667580.0|651780.0|635782.0|619982.0|604182.0|588184.0|572186.0|556188.0|540388.0|524390.0|508590.0|492790.0|476792.0|460992.0|445192.0|429392.0|413394.0|397396.0|381596.0|365796.0|349798.0|333998.0|318198.0|302200.0|286400.0|270600.0|262601.0|254701.0|246801.0|238901.0|231001.0|215003.0|199005.0|183007.0|167207.0|151209.0|135409.0|119609.0|103809.0|87811.0|72011.0|56211.0|40213.0</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>44.38|51.63|56.91|60.43|98.82|98.82|101.36|103.92|147.37|147.37|150.61|150.61|153.86|157.14|160.43|163.74|167.07|170.42|173.78|177.16|180.99|180.99|184.40|184.40|187.84|191.29|191.29|191.29|194.75|194.75|194.75|198.23|201.73|201.73|201.73|205.24|205.24|204.80|209.64|208.32|216.30|216.75|221.21|221.21|221.66|221.66|221.21|216.75|216.75|219.87|219.87|219.42|215.41|215.41|215.41|215.41|215.41|215.41|215.41|211.86|215.41|215.41|215.41|215.41|215.41|215.41|215.41|215.41|215.41|215.41|215.41|215.41|215.41|215.41|215.41|211.86</t>
+        </is>
+      </c>
+      <c r="V6" t="n">
+        <v>377.37</v>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>FEASIBLE</t>
+        </is>
+      </c>
+      <c r="X6" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y6" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>4</v>
+      </c>
+      <c r="AB6" t="n">
+        <v>16384</v>
+      </c>
+      <c r="AC6" t="n">
+        <v>8</v>
+      </c>
+      <c r="AD6" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE6" t="n">
+        <v>3</v>
+      </c>
+      <c r="AF6" t="n">
+        <v>30</v>
+      </c>
+      <c r="AG6" t="n">
+        <v>53.75</v>
+      </c>
+      <c r="AH6" t="n">
+        <v>27</v>
+      </c>
+      <c r="AI6" t="n">
+        <v>45.95</v>
+      </c>
+      <c r="AJ6" t="n">
+        <v>10</v>
+      </c>
+      <c r="AK6" t="n">
+        <v>377.37</v>
+      </c>
+      <c r="AL6" t="inlineStr">
+        <is>
+          <t>FEASIBLE</t>
+        </is>
+      </c>
+      <c r="AM6" t="b">
+        <v>0</v>
+      </c>
+      <c r="AN6" t="n">
+        <v>16384</v>
+      </c>
+      <c r="AO6" t="n">
+        <v>8</v>
+      </c>
+      <c r="AP6" t="n">
+        <v>2</v>
+      </c>
+      <c r="AQ6" t="n">
+        <v>3</v>
+      </c>
+      <c r="AR6" t="n">
+        <v>30</v>
+      </c>
+      <c r="AS6" t="n">
+        <v>53.75</v>
+      </c>
+      <c r="AT6" t="n">
+        <v>27</v>
+      </c>
+      <c r="AU6" t="n">
+        <v>45.95</v>
+      </c>
+      <c r="AV6" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>1500</v>
+      </c>
+      <c r="B7" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>matmul_4x4</t>
+        </is>
+      </c>
+      <c r="D7" t="b">
+        <v>1</v>
+      </c>
+      <c r="E7" t="n">
+        <v>7044</v>
+      </c>
+      <c r="F7" t="n">
+        <v>41.34</v>
+      </c>
+      <c r="G7" t="n">
+        <v>6752</v>
+      </c>
+      <c r="H7" t="n">
+        <v>55.59</v>
+      </c>
+      <c r="I7" t="n">
+        <v>4.15</v>
+      </c>
+      <c r="J7" t="b">
+        <v>0</v>
+      </c>
+      <c r="K7" t="n">
+        <v>6752</v>
+      </c>
+      <c r="L7" t="n">
+        <v>55.59</v>
+      </c>
+      <c r="M7" t="n">
+        <v>4.15</v>
+      </c>
+      <c r="N7" t="b">
+        <v>0</v>
+      </c>
+      <c r="O7" t="b">
+        <v>1</v>
+      </c>
+      <c r="P7" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>3</v>
+      </c>
+      <c r="R7" t="n">
+        <v>485.5</v>
+      </c>
+      <c r="S7" t="n">
+        <v>1444.41</v>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>7044.0|6847.0|6752.0|6752.0</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>41.34|49.87|55.59|55.59</t>
+        </is>
+      </c>
+      <c r="V7" t="n">
+        <v>34.47</v>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>FEASIBLE</t>
+        </is>
+      </c>
+      <c r="X7" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y7" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA7" t="n">
+        <v>2</v>
+      </c>
+      <c r="AB7" t="n">
+        <v>16384</v>
+      </c>
+      <c r="AC7" t="n">
+        <v>4</v>
+      </c>
+      <c r="AD7" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE7" t="n">
+        <v>2</v>
+      </c>
+      <c r="AF7" t="n">
+        <v>6</v>
+      </c>
+      <c r="AG7" t="n">
+        <v>3</v>
+      </c>
+      <c r="AH7" t="n">
+        <v>3</v>
+      </c>
+      <c r="AI7" t="n">
+        <v>25.41</v>
+      </c>
+      <c r="AJ7" t="n">
+        <v>3</v>
+      </c>
+      <c r="AK7" t="n">
+        <v>34.47</v>
+      </c>
+      <c r="AL7" t="inlineStr">
+        <is>
+          <t>FEASIBLE</t>
+        </is>
+      </c>
+      <c r="AM7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AN7" t="n">
+        <v>16384</v>
+      </c>
+      <c r="AO7" t="n">
+        <v>4</v>
+      </c>
+      <c r="AP7" t="n">
+        <v>2</v>
+      </c>
+      <c r="AQ7" t="n">
+        <v>2</v>
+      </c>
+      <c r="AR7" t="n">
+        <v>6</v>
+      </c>
+      <c r="AS7" t="n">
+        <v>3</v>
+      </c>
+      <c r="AT7" t="n">
+        <v>3</v>
+      </c>
+      <c r="AU7" t="n">
+        <v>25.41</v>
+      </c>
+      <c r="AV7" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>1500</v>
+      </c>
+      <c r="B8" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>fc_2layer_4</t>
+        </is>
+      </c>
+      <c r="D8" t="b">
+        <v>1</v>
+      </c>
+      <c r="E8" t="n">
+        <v>10008</v>
+      </c>
+      <c r="F8" t="n">
+        <v>42.64</v>
+      </c>
+      <c r="G8" t="n">
+        <v>534</v>
+      </c>
+      <c r="H8" t="n">
+        <v>56.91</v>
+      </c>
+      <c r="I8" t="n">
+        <v>94.66</v>
+      </c>
+      <c r="J8" t="b">
+        <v>0</v>
+      </c>
+      <c r="K8" t="n">
+        <v>534</v>
+      </c>
+      <c r="L8" t="n">
+        <v>56.91</v>
+      </c>
+      <c r="M8" t="n">
+        <v>94.66</v>
+      </c>
+      <c r="N8" t="b">
+        <v>0</v>
+      </c>
+      <c r="O8" t="b">
+        <v>1</v>
+      </c>
+      <c r="P8" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>6</v>
+      </c>
+      <c r="R8" t="n">
+        <v>178</v>
+      </c>
+      <c r="S8" t="n">
+        <v>1443.09</v>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>10008.0|8068.0|6069.0|4251.0|2434.0|534.0|534.0</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>42.64|49.87|49.00|56.47|56.91|56.91|56.91</t>
+        </is>
+      </c>
+      <c r="V8" t="n">
+        <v>33.47</v>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>FEASIBLE</t>
+        </is>
+      </c>
+      <c r="X8" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y8" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA8" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB8" t="n">
+        <v>16384</v>
+      </c>
+      <c r="AC8" t="n">
+        <v>4</v>
+      </c>
+      <c r="AD8" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE8" t="n">
+        <v>2</v>
+      </c>
+      <c r="AF8" t="n">
+        <v>6</v>
+      </c>
+      <c r="AG8" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="AH8" t="n">
+        <v>4</v>
+      </c>
+      <c r="AI8" t="n">
+        <v>25.41</v>
+      </c>
+      <c r="AJ8" t="n">
+        <v>3</v>
+      </c>
+      <c r="AK8" t="n">
+        <v>33.47</v>
+      </c>
+      <c r="AL8" t="inlineStr">
+        <is>
+          <t>FEASIBLE</t>
+        </is>
+      </c>
+      <c r="AM8" t="b">
+        <v>0</v>
+      </c>
+      <c r="AN8" t="n">
+        <v>16384</v>
+      </c>
+      <c r="AO8" t="n">
+        <v>4</v>
+      </c>
+      <c r="AP8" t="n">
+        <v>2</v>
+      </c>
+      <c r="AQ8" t="n">
+        <v>2</v>
+      </c>
+      <c r="AR8" t="n">
+        <v>6</v>
+      </c>
+      <c r="AS8" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="AT8" t="n">
+        <v>4</v>
+      </c>
+      <c r="AU8" t="n">
+        <v>25.41</v>
+      </c>
+      <c r="AV8" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>1500</v>
+      </c>
+      <c r="B9" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>fc_2layer_8</t>
+        </is>
+      </c>
+      <c r="D9" t="b">
+        <v>1</v>
+      </c>
+      <c r="E9" t="n">
+        <v>26012</v>
+      </c>
+      <c r="F9" t="n">
+        <v>44.38</v>
+      </c>
+      <c r="G9" t="n">
+        <v>958</v>
+      </c>
+      <c r="H9" t="n">
+        <v>77.3</v>
+      </c>
+      <c r="I9" t="n">
+        <v>96.31999999999999</v>
+      </c>
+      <c r="J9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K9" t="n">
+        <v>958</v>
+      </c>
+      <c r="L9" t="n">
+        <v>77.3</v>
+      </c>
+      <c r="M9" t="n">
+        <v>96.31999999999999</v>
+      </c>
+      <c r="N9" t="b">
+        <v>0</v>
+      </c>
+      <c r="O9" t="b">
+        <v>1</v>
+      </c>
+      <c r="P9" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>13</v>
+      </c>
+      <c r="R9" t="n">
+        <v>140.9</v>
+      </c>
+      <c r="S9" t="n">
+        <v>1422.7</v>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>26012.0|24072.0|22156.0|20157.0|18158.0|16258.0|14358.0|12458.0|10558.0|6658.0|4758.0|2858.0|958.0|958.0</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>44.38|51.63|58.68|58.68|56.91|56.91|77.74|77.74|79.05|79.05|80.81|80.81|77.30|77.30</t>
+        </is>
+      </c>
+      <c r="V9" t="n">
+        <v>74.18000000000001</v>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>FEASIBLE</t>
+        </is>
+      </c>
+      <c r="X9" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y9" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA9" t="n">
+        <v>4</v>
+      </c>
+      <c r="AB9" t="n">
+        <v>16384</v>
+      </c>
+      <c r="AC9" t="n">
+        <v>5</v>
+      </c>
+      <c r="AD9" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE9" t="n">
+        <v>2</v>
+      </c>
+      <c r="AF9" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="AG9" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="AH9" t="n">
+        <v>5</v>
+      </c>
+      <c r="AI9" t="n">
+        <v>30.28</v>
+      </c>
+      <c r="AJ9" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="AK9" t="n">
+        <v>74.18000000000001</v>
+      </c>
+      <c r="AL9" t="inlineStr">
+        <is>
+          <t>FEASIBLE</t>
+        </is>
+      </c>
+      <c r="AM9" t="b">
+        <v>0</v>
+      </c>
+      <c r="AN9" t="n">
+        <v>16384</v>
+      </c>
+      <c r="AO9" t="n">
+        <v>5</v>
+      </c>
+      <c r="AP9" t="n">
+        <v>2</v>
+      </c>
+      <c r="AQ9" t="n">
+        <v>2</v>
+      </c>
+      <c r="AR9" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="AS9" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="AT9" t="n">
+        <v>5</v>
+      </c>
+      <c r="AU9" t="n">
+        <v>30.28</v>
+      </c>
+      <c r="AV9" t="n">
+        <v>5.25</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>1500</v>
+      </c>
+      <c r="B10" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>fc_3layer_4</t>
+        </is>
+      </c>
+      <c r="D10" t="b">
+        <v>1</v>
+      </c>
+      <c r="E10" t="n">
+        <v>100013</v>
+      </c>
+      <c r="F10" t="n">
+        <v>42.64</v>
+      </c>
+      <c r="G10" t="n">
+        <v>10659</v>
+      </c>
+      <c r="H10" t="n">
+        <v>119.09</v>
+      </c>
+      <c r="I10" t="n">
+        <v>89.34</v>
+      </c>
+      <c r="J10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K10" t="n">
+        <v>10659</v>
+      </c>
+      <c r="L10" t="n">
+        <v>119.09</v>
+      </c>
+      <c r="M10" t="n">
+        <v>89.34</v>
+      </c>
+      <c r="N10" t="b">
+        <v>0</v>
+      </c>
+      <c r="O10" t="b">
+        <v>1</v>
+      </c>
+      <c r="P10" t="n">
+        <v>47</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>48</v>
+      </c>
+      <c r="R10" t="n">
+        <v>161098.1</v>
+      </c>
+      <c r="S10" t="n">
+        <v>1380.91</v>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>100013.0|98073.0|96074.0|94257.0|92439.0|90440.0|88441.0|86442.0|84443.0|82444.0|80445.0|80445.0|78446.0|76546.0|74646.0|72746.0|70846.0|68946.0|67046.0|65146.0|63246.0|61346.0|59347.0|57348.0|55349.0|53350.0|51450.0|49451.0|47551.0|45651.0|43751.0|41752.0|39753.0|37754.0|35854.0|33954.0|32054.0|30154.0|28155.0|26156.0|24157.0|22158.0|20258.0|18358.0|16458.0|14459.0|12559.0|10659.0|10659.0</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>42.64|49.87|49.00|77.74|75.57|79.05|81.25|83.46|85.68|87.92|90.17|90.17|92.43|94.71|97.00|100.23|102.54|104.87|107.22|109.57|111.93|111.93|114.31|114.31|118.13|120.53|118.13|120.53|118.13|115.74|114.31|117.65|120.05|122.46|120.05|120.05|116.69|116.69|119.09|121.49|123.91|126.34|123.91|123.91|121.49|123.91|121.49|119.09|119.09</t>
+        </is>
+      </c>
+      <c r="V10" t="n">
+        <v>179.3</v>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>FEASIBLE</t>
+        </is>
+      </c>
+      <c r="X10" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y10" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA10" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB10" t="n">
+        <v>16384</v>
+      </c>
+      <c r="AC10" t="n">
+        <v>5</v>
+      </c>
+      <c r="AD10" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE10" t="n">
+        <v>2</v>
+      </c>
+      <c r="AF10" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="AG10" t="n">
+        <v>28.5</v>
+      </c>
+      <c r="AH10" t="n">
+        <v>23</v>
+      </c>
+      <c r="AI10" t="n">
+        <v>30.28</v>
+      </c>
+      <c r="AJ10" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="AK10" t="n">
+        <v>179.3</v>
+      </c>
+      <c r="AL10" t="inlineStr">
+        <is>
+          <t>FEASIBLE</t>
+        </is>
+      </c>
+      <c r="AM10" t="b">
+        <v>0</v>
+      </c>
+      <c r="AN10" t="n">
+        <v>16384</v>
+      </c>
+      <c r="AO10" t="n">
+        <v>5</v>
+      </c>
+      <c r="AP10" t="n">
+        <v>2</v>
+      </c>
+      <c r="AQ10" t="n">
+        <v>2</v>
+      </c>
+      <c r="AR10" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="AS10" t="n">
+        <v>28.5</v>
+      </c>
+      <c r="AT10" t="n">
+        <v>23</v>
+      </c>
+      <c r="AU10" t="n">
+        <v>30.28</v>
+      </c>
+      <c r="AV10" t="n">
+        <v>5.25</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>1500</v>
+      </c>
+      <c r="B11" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>matmul_8x8</t>
+        </is>
+      </c>
+      <c r="D11" t="b">
+        <v>1</v>
+      </c>
+      <c r="E11" t="n">
+        <v>135014</v>
+      </c>
+      <c r="F11" t="n">
+        <v>44.38</v>
+      </c>
+      <c r="G11" t="n">
+        <v>1359</v>
+      </c>
+      <c r="H11" t="n">
+        <v>111.7</v>
+      </c>
+      <c r="I11" t="n">
+        <v>98.98999999999999</v>
+      </c>
+      <c r="J11" t="b">
+        <v>0</v>
+      </c>
+      <c r="K11" t="n">
+        <v>1359</v>
+      </c>
+      <c r="L11" t="n">
+        <v>111.7</v>
+      </c>
+      <c r="M11" t="n">
+        <v>98.98999999999999</v>
+      </c>
+      <c r="N11" t="b">
+        <v>0</v>
+      </c>
+      <c r="O11" t="b">
+        <v>1</v>
+      </c>
+      <c r="P11" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>14</v>
+      </c>
+      <c r="R11" t="n">
+        <v>31858.4</v>
+      </c>
+      <c r="S11" t="n">
+        <v>1388.3</v>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>135014.0|134169.0|132237.0|128353.0|120453.0|112553.0|96555.0|88556.0|80557.0|64757.0|48957.0|32959.0|17159.0|1359.0|1359.0</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>44.38|51.63|56.91|60.43|98.82|98.82|101.36|105.64|103.92|106.50|109.09|109.09|111.70|111.70|111.70</t>
+        </is>
+      </c>
+      <c r="V11" t="n">
+        <v>151.69</v>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>FEASIBLE</t>
+        </is>
+      </c>
+      <c r="X11" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y11" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA11" t="n">
+        <v>4</v>
+      </c>
+      <c r="AB11" t="n">
+        <v>16384</v>
+      </c>
+      <c r="AC11" t="n">
+        <v>6</v>
+      </c>
+      <c r="AD11" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE11" t="n">
+        <v>3</v>
+      </c>
+      <c r="AF11" t="n">
+        <v>18</v>
+      </c>
+      <c r="AG11" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="AH11" t="n">
+        <v>10</v>
+      </c>
+      <c r="AI11" t="n">
+        <v>35.32</v>
+      </c>
+      <c r="AJ11" t="n">
+        <v>6</v>
+      </c>
+      <c r="AK11" t="n">
+        <v>151.69</v>
+      </c>
+      <c r="AL11" t="inlineStr">
+        <is>
+          <t>FEASIBLE</t>
+        </is>
+      </c>
+      <c r="AM11" t="b">
+        <v>0</v>
+      </c>
+      <c r="AN11" t="n">
+        <v>16384</v>
+      </c>
+      <c r="AO11" t="n">
+        <v>6</v>
+      </c>
+      <c r="AP11" t="n">
+        <v>2</v>
+      </c>
+      <c r="AQ11" t="n">
+        <v>3</v>
+      </c>
+      <c r="AR11" t="n">
+        <v>18</v>
+      </c>
+      <c r="AS11" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="AT11" t="n">
+        <v>10</v>
+      </c>
+      <c r="AU11" t="n">
+        <v>35.32</v>
+      </c>
+      <c r="AV11" t="n">
         <v>6</v>
       </c>
     </row>

</xml_diff>